<commit_message>
add machine learning porttion
</commit_message>
<xml_diff>
--- a/LAB/Flat_Price_Multiple_Linear_Regression_100 (1).xlsx
+++ b/LAB/Flat_Price_Multiple_Linear_Regression_100 (1).xlsx
@@ -1,21 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BWU\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6AD979A1-7927-437D-BFB5-F7A7FF6E7B70}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Flat_Data" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Flat_Data" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -58,22 +49,23 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -94,16 +86,16 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -116,13 +108,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -177,7 +169,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -210,26 +202,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -262,23 +237,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -313,20 +271,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -448,23 +402,63 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G101"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="21" style="2" customWidth="1"/>
-    <col min="5" max="5" width="20.85546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="20.42578125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="19.7109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="16.857142857142858" customWidth="1"/>
+    <col min="2" max="2" width="28.142857142857142" customWidth="1"/>
+    <col min="3" max="3" width="18.285714285714285" customWidth="1"/>
+    <col min="4" max="4" width="21" customWidth="1"/>
+    <col min="5" max="5" width="20.857142857142858" customWidth="1"/>
+    <col min="6" max="6" width="20.428571428571427" customWidth="1"/>
+    <col min="7" max="7" width="19.714285714285715" customWidth="1"/>
+    <col min="8" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2792,5 +2786,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>